<commit_message>
feat: finalize female analysis report with resolved names and multi-scale metric annotations
</commit_message>
<xml_diff>
--- a/data/results/female_analysis/female_top200_clustering.xlsx
+++ b/data/results/female_analysis/female_top200_clustering.xlsx
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>my mother</t>
+          <t>my mother (The_Distant_Land_of_My_Father)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -493,7 +493,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>May (Shanghai_Girls)</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -523,7 +523,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Magic Gourd</t>
+          <t>Magic Gourd (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -553,7 +553,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pearl</t>
+          <t>Pearl (Peach_Blossom_Pavillion)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -583,7 +583,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>my mother</t>
+          <t>my mother (Sour_Heart)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -613,7 +613,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Claire</t>
+          <t>Claire (Rabbit_Moon)</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -643,7 +643,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Yu</t>
+          <t>Yu (Death_of_a_Red_Heroine)</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -673,7 +673,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hannah</t>
+          <t>Hannah (The_Far_Side_of_the_Sky_Adler_Family_1)</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -703,7 +703,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mother</t>
+          <t>Mother (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -733,7 +733,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sparrow</t>
+          <t>Sparrow (The_Library_of_Legends)</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -763,7 +763,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>my mother</t>
+          <t>my mother (Dragon_Springs_Road)</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -793,7 +793,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Joy</t>
+          <t>Joy (Shanghai_Girls)</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -823,7 +823,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>JinJin</t>
+          <t>JinJin (My_Favourite_Wife)</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -853,7 +853,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Caitlin</t>
+          <t>Caitlin (Jack_of_Spies)</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -883,7 +883,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Holly</t>
+          <t>Holly (My_Favourite_Wife)</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -913,7 +913,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>my grandmother</t>
+          <t>my grandmother (The_Distant_Land_of_My_Father)</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -943,7 +943,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Yan</t>
+          <t>Yan (All_the_Flowers_in_Shanghai)</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -973,7 +973,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mama</t>
+          <t>Mama (Peach_Blossom_Pavillion)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1003,7 +1003,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gigi</t>
+          <t>Gigi (Shanghai_Immortal)</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1033,7 +1033,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>Sunny (Song_of_the_Exile)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1063,7 +1063,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Xu</t>
+          <t>Xu (Blue_Hunger_Viola_Di_Grado)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1093,7 +1093,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Alice (The_Shanghai_Moon)</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1123,7 +1123,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mama</t>
+          <t>Mama (Shanghai_Girls)</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1153,7 +1153,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Anjuin</t>
+          <t>Anjuin (Dragon_Springs_Road)</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1183,7 +1183,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Meirong</t>
+          <t>Meirong (The_Library_of_Legends)</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1213,7 +1213,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mother</t>
+          <t>Mother (Peach_Blossom_Pavillion)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1243,7 +1243,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>my mom</t>
+          <t>my mom (Sour_Heart)</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1273,7 +1273,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Fox</t>
+          <t>Fox (Dragon_Springs_Road)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1303,7 +1303,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Mary (The_Shanghai_Moon)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1333,7 +1333,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Anna (Dragon_Springs_Road)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1363,7 +1363,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mei</t>
+          <t>Mei (The_Shanghai_Factor)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1393,7 +1393,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jia - Li</t>
+          <t>Jia - Li (The_Far_Side_of_the_Sky_Adler_Family_1)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1423,7 +1423,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ping Mei</t>
+          <t>Ping Mei (Dragon_Springs_Road)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1453,7 +1453,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>her mother</t>
+          <t>her mother (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1483,7 +1483,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Grandmother Yang</t>
+          <t>Grandmother Yang (Dragon_Springs_Road)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1513,7 +1513,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Alice (The_Shanghai_Factor)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1543,7 +1543,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mother</t>
+          <t>Mother (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1573,7 +1573,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Anne</t>
+          <t>Anne (The_Map_of_Lost_Memories)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1603,7 +1603,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pomelo</t>
+          <t>Pomelo (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1633,7 +1633,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Jinling</t>
+          <t>Jinling (The_Painter_From_Shanghai)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1663,7 +1663,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Rose</t>
+          <t>Rose (What_We_Were_Promised)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1693,7 +1693,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Granny</t>
+          <t>Granny (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1723,7 +1723,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mrs. Shen</t>
+          <t>Mrs. Shen (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1753,7 +1753,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>his mother</t>
+          <t>his mother (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1783,7 +1783,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Madam Zhang</t>
+          <t>Madam Zhang (All_the_Flowers_in_Shanghai)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1813,7 +1813,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>my grandmother</t>
+          <t>my grandmother (Sour_Heart)</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1843,7 +1843,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Qian</t>
+          <t>Qian (Shanghai_Redemption)</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1873,7 +1873,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Leah</t>
+          <t>Leah (Shanghai)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1903,7 +1903,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Miss Schwartz</t>
+          <t>Miss Schwartz (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1933,7 +1933,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Fang Rong</t>
+          <t>Fang Rong (Peach_Blossom_Pavillion)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1963,7 +1963,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Fairlynn</t>
+          <t>Fairlynn (Becoming_Madame_Mao)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1993,7 +1993,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>the woman</t>
+          <t>the woman (Five_Star_Billionaire)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2023,7 +2023,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Florence</t>
+          <t>Florence (Shanghai)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -2053,7 +2053,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Shanshan</t>
+          <t>Shanshan (Dont_Cry_Tai_Lake)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2083,7 +2083,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Yanyan</t>
+          <t>Yanyan (Five_Star_Billionaire)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -2113,7 +2113,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Miss Morris</t>
+          <t>Miss Morris (Dragon_Springs_Road)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2143,7 +2143,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Madam Li</t>
+          <t>Madam Li (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2173,7 +2173,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Peiqin</t>
+          <t>Peiqin (When_Red_Is_Black)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2203,7 +2203,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Leah</t>
+          <t>Leah (Dragon_Springs_Road)</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2233,7 +2233,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>The woman</t>
+          <t>The woman (The_Master_of_Rain)</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2263,7 +2263,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Clara</t>
+          <t>Clara (The_Far_Side_of_the_Sky_Adler_Family_1)</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2293,7 +2293,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Devlin</t>
+          <t>Devlin (My_Favourite_Wife)</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2323,7 +2323,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Yu - ying</t>
+          <t>Yu - ying (The_Binding_Chair)</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2353,7 +2353,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Francine</t>
+          <t>Francine (Sour_Heart)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2383,7 +2383,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Peiqin</t>
+          <t>Peiqin (Shanghai_Redemption)</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2413,7 +2413,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Nancy (My_Favourite_Wife)</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2443,7 +2443,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Arthur (The_Binding_Chair)</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2473,7 +2473,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Alice (My_Favourite_Wife)</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2503,7 +2503,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Taitai</t>
+          <t>Taitai (What_We_Were_Promised)</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2533,7 +2533,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Peiqin</t>
+          <t>Peiqin (Death_of_a_Red_Heroine)</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2563,7 +2563,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Irina</t>
+          <t>Irina (Shanghai)</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2593,7 +2593,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Fanpin</t>
+          <t>Fanpin (Sour_Heart)</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2623,7 +2623,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Lianping</t>
+          <t>Lianping (Enigma_of_China)</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2653,7 +2653,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Old Hunter</t>
+          <t>Old Hunter (Shanghai_Redemption)</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2683,7 +2683,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>the woman</t>
+          <t>the woman (These_Violent_Delights)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2713,7 +2713,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Azure</t>
+          <t>Azure (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -2743,7 +2743,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Simone (The_Map_of_Lost_Memories)</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2773,7 +2773,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Manzhen</t>
+          <t>Manzhen (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2803,7 +2803,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Alice (The_Binding_Chair)</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2833,7 +2833,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Natasha</t>
+          <t>Natasha (The_Master_of_Rain)</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2863,7 +2863,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Becca</t>
+          <t>Becca (My_Favourite_Wife)</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2893,7 +2893,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Nina</t>
+          <t>Nina (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2923,7 +2923,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Kathleen</t>
+          <t>Kathleen (These_Violent_Delights)</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -2953,7 +2953,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Li</t>
+          <t>Li (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2983,7 +2983,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Yumi</t>
+          <t>Yumi (Shanghailanders)</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -3013,7 +3013,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Tsuizhi</t>
+          <t>Tsuizhi (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -3043,7 +3043,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Catherine</t>
+          <t>Catherine (A_Loyal_Character_Dancer)</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -3073,7 +3073,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Manlu</t>
+          <t>Manlu (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -3103,7 +3103,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>my mother</t>
+          <t>my mother (Dreams_of_Joy)</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -3133,7 +3133,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>her mother</t>
+          <t>her mother (The_Library_of_Legends)</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -3163,7 +3163,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Clothilde</t>
+          <t>Clothilde (The_Map_of_Lost_Memories)</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -3193,7 +3193,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Sister</t>
+          <t>Sister (All_the_Flowers_in_Shanghai)</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -3223,7 +3223,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Flora</t>
+          <t>Flora (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -3253,7 +3253,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Ma</t>
+          <t>Ma (All_the_Flowers_in_Shanghai)</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -3283,7 +3283,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Jenmei</t>
+          <t>Jenmei (The_Library_of_Legends)</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -3313,7 +3313,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Golden Dove</t>
+          <t>Golden Dove (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -3343,7 +3343,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Mei</t>
+          <t>Mei (Rabbit_Moon)</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -3373,7 +3373,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>his wife</t>
+          <t>his wife (My_Favourite_Wife)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -3403,7 +3403,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Lady Soo</t>
+          <t>Lady Soo (Shanghai_Immortal)</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -3433,7 +3433,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>his daughter</t>
+          <t>his daughter (My_Favourite_Wife)</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -3463,7 +3463,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Amy</t>
+          <t>Amy (The_Risk_Agent)</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -3493,7 +3493,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Niang Niang</t>
+          <t>Niang Niang (Shanghai_Immortal)</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -3523,7 +3523,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>May (Dreams_of_Joy)</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -3553,7 +3553,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Kate</t>
+          <t>Kate (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -3583,7 +3583,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Leilani</t>
+          <t>Leilani (Song_of_the_Exile)</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -3613,7 +3613,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>the girl</t>
+          <t>the girl (Five_Star_Billionaire)</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -3643,7 +3643,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Peiqin</t>
+          <t>Peiqin (Red_Mandarin_Dress_Inspector_Chen_Cao_5)</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -3673,7 +3673,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Mao</t>
+          <t>Mao (Becoming_Madame_Mao)</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -3703,7 +3703,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Wen</t>
+          <t>Wen (A_Loyal_Character_Dancer)</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -3733,7 +3733,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Jiao</t>
+          <t>Jiao (The_Mao_Case)</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -3763,7 +3763,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Tao</t>
+          <t>Tao (Dreams_of_Joy)</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -3793,7 +3793,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Kumei</t>
+          <t>Kumei (Dreams_of_Joy)</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -3823,7 +3823,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>my daughter</t>
+          <t>my daughter (Dreams_of_Joy)</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -3853,7 +3853,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Grace (Rabbit_Moon)</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -3883,7 +3883,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>a woman</t>
+          <t>a woman (Song_of_the_Exile)</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -3913,7 +3913,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>my mother</t>
+          <t>my mother (The_Library_of_Legends)</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -3943,7 +3943,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Rosalie</t>
+          <t>Rosalie (The_Shanghai_Moon)</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -3973,7 +3973,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>The top girl</t>
+          <t>The top girl (The_Painter_From_Shanghai)</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -4003,7 +4003,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Mother</t>
+          <t>Mother (The_Shanghai_Factor)</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -4033,7 +4033,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Rosalita</t>
+          <t>Rosalita (My_Favourite_Wife)</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -4063,7 +4063,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Godmother</t>
+          <t>Godmother (The_Painter_From_Shanghai)</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -4093,7 +4093,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Yen - yen</t>
+          <t>Yen - yen (Shanghai_Girls)</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -4123,7 +4123,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Magdalena</t>
+          <t>Magdalena (The_Shanghai_Factor)</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -4153,7 +4153,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>my mother</t>
+          <t>my mother (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -4183,7 +4183,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Yoko</t>
+          <t>Yoko (Shanghailanders)</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -4213,7 +4213,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Karen</t>
+          <t>Karen (What_We_Were_Promised)</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -4243,7 +4243,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Joy</t>
+          <t>Joy (Dreams_of_Joy)</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -4273,7 +4273,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Esther</t>
+          <t>Esther (The_Far_Side_of_the_Sky_Adler_Family_1)</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -4303,7 +4303,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Penelope</t>
+          <t>Penelope (The_Master_of_Rain)</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -4333,7 +4333,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Mutti</t>
+          <t>Mutti (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -4363,7 +4363,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>my daughter</t>
+          <t>my daughter (Shanghai_Girls)</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -4393,7 +4393,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Eleanor</t>
+          <t>Eleanor (The_Binding_Chair)</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -4423,7 +4423,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Rosalind</t>
+          <t>Rosalind (These_Violent_Delights)</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -4453,7 +4453,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Yong</t>
+          <t>Yong (Dreams_of_Joy)</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -4483,7 +4483,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Yuliang</t>
+          <t>Yuliang (The_Painter_From_Shanghai)</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -4513,7 +4513,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Yin</t>
+          <t>Yin (When_Red_Is_Black)</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -4543,7 +4543,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>the girl</t>
+          <t>the girl (Becoming_Madame_Mao)</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -4573,7 +4573,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Pearl</t>
+          <t>Pearl (Peach_Blossom_Pavillion)</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -4603,7 +4603,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Lena</t>
+          <t>Lena (The_Master_of_Rain)</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -4633,7 +4633,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Liu</t>
+          <t>Liu (Dont_Cry_Tai_Lake)</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -4663,7 +4663,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Guan</t>
+          <t>Guan (Death_of_a_Red_Heroine)</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -4693,7 +4693,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Zhou</t>
+          <t>Zhou (Enigma_of_China)</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -4723,7 +4723,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Xiuqing</t>
+          <t>Xiuqing (The_Painter_From_Shanghai)</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -4753,7 +4753,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>my sister</t>
+          <t>my sister (Shanghai_Girls)</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -4783,7 +4783,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Violet</t>
+          <t>Violet (The_Valley_of_Amazement)</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -4813,7 +4813,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>the woman</t>
+          <t>the woman (The_Painter_From_Shanghai)</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -4843,7 +4843,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Lan Ping</t>
+          <t>Lan Ping (Becoming_Madame_Mao)</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -4873,7 +4873,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>my mother</t>
+          <t>my mother (Peach_Blossom_Pavillion)</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -4903,7 +4903,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>the girl</t>
+          <t>the girl (The_Painter_From_Shanghai)</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -4933,7 +4933,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>An</t>
+          <t>An (A_Case_of_Two_Cities)</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -4963,7 +4963,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>my mother</t>
+          <t>my mother (The_Shanghai_Moon)</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -4993,7 +4993,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Opa</t>
+          <t>Opa (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -5023,7 +5023,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>her daughter</t>
+          <t>her daughter (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -5053,7 +5053,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Mi</t>
+          <t>Mi (Dont_Cry_Tai_Lake)</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -5083,7 +5083,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (Shanghai_Girls)</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -5113,7 +5113,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (The_Map_of_Lost_Memories)</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -5143,7 +5143,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (Death_of_a_Red_Heroine)</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -5173,7 +5173,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (Song_of_the_Exile)</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -5203,7 +5203,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (Shanghailanders)</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -5233,7 +5233,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -5263,7 +5263,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -5293,7 +5293,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (When_Red_Is_Black)</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -5323,7 +5323,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (Rabbit_Moon)</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -5353,7 +5353,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (The_Binding_Chair)</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -5383,7 +5383,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Xiang Xiang</t>
+          <t>Xiang Xiang (Peach_Blossom_Pavillion)</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -5413,7 +5413,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (These_Violent_Delights)</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -5443,7 +5443,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Mama</t>
+          <t>Mama (The_Shanghai_Moon)</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -5473,7 +5473,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (Sour_Heart)</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -5503,7 +5503,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Juliette</t>
+          <t>Juliette (These_Violent_Delights)</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -5533,7 +5533,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (Dragon_Springs_Road)</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -5563,7 +5563,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Romy</t>
+          <t>Romy (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -5593,7 +5593,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Character_0</t>
+          <t>Character_0 (Blue_Hunger_Viola_Di_Grado)</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -5623,7 +5623,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>Sunny (The_Far_Side_of_the_Sky_Adler_Family_1)</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -5653,7 +5653,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Phoebe</t>
+          <t>Phoebe (Five_Star_Billionaire)</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -5683,7 +5683,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>May (The_Binding_Chair)</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -5713,7 +5713,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Grace</t>
+          <t>Grace (The_Risk_Agent)</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -5743,7 +5743,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Lindsey</t>
+          <t>Lindsey (Rabbit_Moon)</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -5773,7 +5773,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Lian</t>
+          <t>Lian (The_Library_of_Legends)</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -5803,7 +5803,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Sunny</t>
+          <t>Sunny (What_We_Were_Promised)</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -5833,7 +5833,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Yinghui</t>
+          <t>Yinghui (Five_Star_Billionaire)</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -5863,7 +5863,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Mrs. Gu</t>
+          <t>Mrs. Gu (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -5893,7 +5893,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Malia</t>
+          <t>Malia (Song_of_the_Exile)</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -5923,7 +5923,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Eko</t>
+          <t>Eko (Shanghailanders)</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -5953,7 +5953,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Suzanne</t>
+          <t>Suzanne (The_Binding_Chair)</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -5983,7 +5983,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Song</t>
+          <t>Song (Night_in_Shanghai)</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -6013,7 +6013,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Kiko</t>
+          <t>Kiko (Shanghailanders)</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -6043,7 +6043,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Chen</t>
+          <t>Chen (When_Red_Is_Black)</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -6073,7 +6073,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Ah Bao</t>
+          <t>Ah Bao (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -6103,7 +6103,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Manzhen</t>
+          <t>Manzhen (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -6133,7 +6133,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Alisa</t>
+          <t>Alisa (These_Violent_Delights)</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -6163,7 +6163,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Catherine</t>
+          <t>Catherine (A_Case_of_Two_Cities)</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -6193,7 +6193,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Phoebe</t>
+          <t>Phoebe (Five_Star_Billionaire)</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -6223,7 +6223,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Oma</t>
+          <t>Oma (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -6253,7 +6253,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Peiqin</t>
+          <t>Peiqin (A_Case_of_Two_Cities)</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -6283,7 +6283,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Eleanor</t>
+          <t>Eleanor (The_Binding_Chair)</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -6313,7 +6313,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>her grandmother</t>
+          <t>her grandmother (The_Song_of_the_Jade_Lily)</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -6343,7 +6343,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>the girl</t>
+          <t>the girl (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -6373,7 +6373,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>the woman</t>
+          <t>the woman (Song_of_the_Exile)</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -6403,7 +6403,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Mrs. Hsu</t>
+          <t>Mrs. Hsu (Half_a_Lifelong_Romance)</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -6433,7 +6433,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Lily</t>
+          <t>Lily (Rabbit_Moon)</t>
         </is>
       </c>
       <c r="B201" t="n">

</xml_diff>